<commit_message>
DungeonTransferConfig英文配置加c,不然启动机器人会报错？？ 2025-07-21 15:39:45.5286 configType:  DungeonTransferConfigCategory    at ET.ConfigComponentSystem.LoadOneInThread(ConfigComponent self, Type configType, Dictionary`2 configBytes) in H:\GitWeiJing\Unity\Assets\Hotfix\Module\Config\ConfigComponentSystem.cs:line 84
</commit_message>
<xml_diff>
--- a/Excel/DungeonTransferConfig.xlsx
+++ b/Excel/DungeonTransferConfig.xlsx
@@ -27,7 +27,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="256">
+  <si>
+    <t>c</t>
+  </si>
   <si>
     <t>Id</t>
   </si>
@@ -1878,7 +1881,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="C3:S66"/>
+  <dimension ref="C2:S66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="21.125" style="1" customWidth="1"/>
@@ -1891,73 +1894,78 @@
     <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="5:5">
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
     <row r="3" spans="3:9">
       <c r="C3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="3:9">
       <c r="C4" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="3:9">
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="3:9">
@@ -1965,10 +1973,10 @@
         <v>1001</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="4">
         <v>10001</v>
@@ -1977,10 +1985,10 @@
         <v>1</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="3:19">
@@ -1988,10 +1996,10 @@
         <v>1002</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F7" s="6">
         <v>10002</v>
@@ -2000,10 +2008,10 @@
         <v>1</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K7" s="1">
         <v>15200</v>
@@ -2036,10 +2044,10 @@
         <v>1003</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="4">
         <v>10003</v>
@@ -2048,10 +2056,10 @@
         <v>5</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K8" s="1">
         <v>16292</v>
@@ -2084,10 +2092,10 @@
         <v>1004</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" s="4">
         <v>10004</v>
@@ -2096,10 +2104,10 @@
         <v>1</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K9" s="1">
         <v>15400</v>
@@ -2132,10 +2140,10 @@
         <v>1005</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F10" s="4">
         <v>10005</v>
@@ -2144,10 +2152,10 @@
         <v>5</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K10" s="1">
         <v>14400</v>
@@ -2180,10 +2188,10 @@
         <v>1006</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F11" s="4">
         <v>10006</v>
@@ -2192,10 +2200,10 @@
         <v>12</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K11" s="1">
         <v>16800</v>
@@ -2228,10 +2236,10 @@
         <v>1007</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F12" s="4">
         <v>10007</v>
@@ -2240,10 +2248,10 @@
         <v>8</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K12" s="1">
         <v>14300</v>
@@ -2276,10 +2284,10 @@
         <v>1008</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F13" s="4">
         <v>10008</v>
@@ -2288,10 +2296,10 @@
         <v>1</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K13" s="1">
         <v>14400</v>
@@ -2324,10 +2332,10 @@
         <v>1009</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F14" s="4">
         <v>10001</v>
@@ -2336,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K14" s="1">
         <v>7670</v>
@@ -2372,10 +2380,10 @@
         <v>1010</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F15" s="6">
         <v>10002</v>
@@ -2384,10 +2392,10 @@
         <v>1</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K15" s="1">
         <v>15819</v>
@@ -2420,10 +2428,10 @@
         <v>1011</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F16" s="4">
         <v>10004</v>
@@ -2432,10 +2440,10 @@
         <v>1</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K16" s="1">
         <v>25700</v>
@@ -2468,10 +2476,10 @@
         <v>1012</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F17" s="4">
         <v>10008</v>
@@ -2480,10 +2488,10 @@
         <v>1</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K17" s="1">
         <v>20300</v>
@@ -2516,10 +2524,10 @@
         <v>1013</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F18" s="4">
         <v>10004</v>
@@ -2528,10 +2536,10 @@
         <v>1</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K18" s="1">
         <v>26100</v>
@@ -2564,10 +2572,10 @@
         <v>1014</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F19" s="4">
         <v>10007</v>
@@ -2576,10 +2584,10 @@
         <v>1</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K19" s="1">
         <v>25310</v>
@@ -2612,10 +2620,10 @@
         <v>2001</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F20" s="4">
         <v>20001</v>
@@ -2624,7 +2632,7 @@
         <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I20" s="9"/>
       <c r="K20" s="1">
@@ -2658,10 +2666,10 @@
         <v>2002</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F21" s="4">
         <v>20002</v>
@@ -2670,10 +2678,10 @@
         <v>15</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K21" s="1">
         <v>15259</v>
@@ -2706,10 +2714,10 @@
         <v>2003</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F22" s="4">
         <v>20003</v>
@@ -2718,10 +2726,10 @@
         <v>15</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K22" s="1">
         <v>15756</v>
@@ -2754,10 +2762,10 @@
         <v>2004</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F23" s="4">
         <v>20004</v>
@@ -2766,10 +2774,10 @@
         <v>15</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K23" s="1">
         <v>14613</v>
@@ -2802,10 +2810,10 @@
         <v>2005</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F24" s="4">
         <v>20005</v>
@@ -2814,10 +2822,10 @@
         <v>15</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K24" s="1">
         <v>21779</v>
@@ -2850,10 +2858,10 @@
         <v>2011</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F25" s="4">
         <v>20001</v>
@@ -2862,10 +2870,10 @@
         <v>15</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K25" s="1">
         <v>2139</v>
@@ -2898,10 +2906,10 @@
         <v>2012</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F26" s="4">
         <v>20002</v>
@@ -2910,10 +2918,10 @@
         <v>15</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K26" s="1">
         <v>5935</v>
@@ -2946,10 +2954,10 @@
         <v>2013</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F27" s="4">
         <v>20001</v>
@@ -2958,10 +2966,10 @@
         <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K27" s="1">
         <v>13404</v>
@@ -2994,10 +3002,10 @@
         <v>2014</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F28" s="4">
         <v>20004</v>
@@ -3006,10 +3014,10 @@
         <v>15</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K28" s="1">
         <v>18734</v>
@@ -3042,10 +3050,10 @@
         <v>3001</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F29" s="4">
         <v>30001</v>
@@ -3054,7 +3062,7 @@
         <v>15</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I29" s="9"/>
       <c r="K29" s="1">
@@ -3088,10 +3096,10 @@
         <v>3002</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F30" s="4">
         <v>30002</v>
@@ -3100,10 +3108,10 @@
         <v>15</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K30" s="1">
         <v>13898</v>
@@ -3136,10 +3144,10 @@
         <v>3003</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F31" s="4">
         <v>30003</v>
@@ -3148,10 +3156,10 @@
         <v>15</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K31" s="1">
         <v>14983</v>
@@ -3184,10 +3192,10 @@
         <v>3004</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F32" s="4">
         <v>30004</v>
@@ -3196,10 +3204,10 @@
         <v>15</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I32" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K32" s="1">
         <v>14000</v>
@@ -3232,10 +3240,10 @@
         <v>3005</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F33" s="4">
         <v>30005</v>
@@ -3244,10 +3252,10 @@
         <v>15</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K33" s="1">
         <v>14372</v>
@@ -3280,10 +3288,10 @@
         <v>3006</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F34" s="4">
         <v>30006</v>
@@ -3292,10 +3300,10 @@
         <v>15</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K34" s="1">
         <v>14883</v>
@@ -3328,10 +3336,10 @@
         <v>3011</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F35" s="4">
         <v>30001</v>
@@ -3340,10 +3348,10 @@
         <v>15</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K35" s="1">
         <v>21591</v>
@@ -3376,10 +3384,10 @@
         <v>3012</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F36" s="4">
         <v>30002</v>
@@ -3388,10 +3396,10 @@
         <v>15</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K36" s="1">
         <v>23656</v>
@@ -3424,10 +3432,10 @@
         <v>3013</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F37" s="4">
         <v>30002</v>
@@ -3436,10 +3444,10 @@
         <v>15</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K37" s="1">
         <v>24258</v>
@@ -3472,10 +3480,10 @@
         <v>3014</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F38" s="4">
         <v>30004</v>
@@ -3484,10 +3492,10 @@
         <v>15</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I38" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K38" s="1">
         <v>16698</v>
@@ -3520,10 +3528,10 @@
         <v>3015</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F39" s="4">
         <v>30005</v>
@@ -3532,10 +3540,10 @@
         <v>15</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K39" s="1">
         <v>25092</v>
@@ -3568,10 +3576,10 @@
         <v>3016</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F40" s="4">
         <v>30006</v>
@@ -3580,10 +3588,10 @@
         <v>16</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="3:19">
@@ -3591,10 +3599,10 @@
         <v>4001</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F41" s="4">
         <v>40001</v>
@@ -3603,7 +3611,7 @@
         <v>15</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I41" s="9"/>
       <c r="K41" s="1">
@@ -3637,10 +3645,10 @@
         <v>4002</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F42" s="4">
         <v>40002</v>
@@ -3649,10 +3657,10 @@
         <v>15</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K42" s="1">
         <v>17650</v>
@@ -3685,10 +3693,10 @@
         <v>4003</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F43" s="4">
         <v>40003</v>
@@ -3697,10 +3705,10 @@
         <v>15</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K43" s="1">
         <v>17670</v>
@@ -3733,10 +3741,10 @@
         <v>4004</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F44" s="4">
         <v>40004</v>
@@ -3745,10 +3753,10 @@
         <v>15</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K44" s="1">
         <v>25645</v>
@@ -3781,10 +3789,10 @@
         <v>4005</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F45" s="4">
         <v>40005</v>
@@ -3793,10 +3801,10 @@
         <v>15</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I45" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K45" s="1">
         <v>14301</v>
@@ -3829,10 +3837,10 @@
         <v>4006</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F46" s="4">
         <v>40006</v>
@@ -3841,10 +3849,10 @@
         <v>15</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K46" s="1">
         <v>14611</v>
@@ -3877,10 +3885,10 @@
         <v>4007</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F47" s="4">
         <v>40007</v>
@@ -3889,10 +3897,10 @@
         <v>15</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K47" s="1">
         <v>24409</v>
@@ -3925,10 +3933,10 @@
         <v>4011</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F48" s="4">
         <v>40001</v>
@@ -3937,10 +3945,10 @@
         <v>15</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K48" s="1">
         <v>22343</v>
@@ -3973,10 +3981,10 @@
         <v>4012</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F49" s="4">
         <v>40001</v>
@@ -3985,10 +3993,10 @@
         <v>15</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K49" s="1">
         <v>22823</v>
@@ -4021,10 +4029,10 @@
         <v>4013</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F50" s="4">
         <v>40003</v>
@@ -4033,10 +4041,10 @@
         <v>15</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K50" s="1">
         <v>15969</v>
@@ -4069,10 +4077,10 @@
         <v>4014</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F51" s="4">
         <v>40004</v>
@@ -4081,10 +4089,10 @@
         <v>15</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K51" s="1">
         <v>15161</v>
@@ -4117,10 +4125,10 @@
         <v>4015</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F52" s="4">
         <v>40006</v>
@@ -4129,10 +4137,10 @@
         <v>15</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K52" s="1">
         <v>28843</v>
@@ -4165,10 +4173,10 @@
         <v>4016</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F53" s="4">
         <v>40002</v>
@@ -4177,10 +4185,10 @@
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K53" s="1">
         <v>20397</v>
@@ -4213,10 +4221,10 @@
         <v>5001</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F54" s="4">
         <v>50001</v>
@@ -4225,7 +4233,7 @@
         <v>15</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K54" s="1">
         <v>231</v>
@@ -4258,10 +4266,10 @@
         <v>5002</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F55" s="4">
         <v>50002</v>
@@ -4270,10 +4278,10 @@
         <v>15</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I55" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K55" s="1">
         <v>15993</v>
@@ -4306,10 +4314,10 @@
         <v>5003</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F56" s="4">
         <v>50003</v>
@@ -4318,10 +4326,10 @@
         <v>15</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K56" s="1">
         <v>15110</v>
@@ -4354,10 +4362,10 @@
         <v>5004</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F57" s="4">
         <v>50004</v>
@@ -4366,10 +4374,10 @@
         <v>15</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K57" s="1">
         <v>14457</v>
@@ -4402,10 +4410,10 @@
         <v>5005</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F58" s="4">
         <v>50005</v>
@@ -4414,10 +4422,10 @@
         <v>15</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K58" s="1">
         <v>3289</v>
@@ -4450,10 +4458,10 @@
         <v>5006</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F59" s="4">
         <v>50006</v>
@@ -4462,10 +4470,10 @@
         <v>15</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K59" s="1">
         <v>38905</v>
@@ -4498,10 +4506,10 @@
         <v>5007</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F60" s="4">
         <v>50007</v>
@@ -4510,10 +4518,10 @@
         <v>15</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K60" s="1">
         <v>38443</v>
@@ -4546,10 +4554,10 @@
         <v>5011</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F61" s="4">
         <v>50001</v>
@@ -4558,10 +4566,10 @@
         <v>15</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K61" s="1">
         <v>7832</v>
@@ -4594,10 +4602,10 @@
         <v>5012</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F62" s="4">
         <v>50002</v>
@@ -4606,10 +4614,10 @@
         <v>15</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K62" s="1">
         <v>13618</v>
@@ -4642,10 +4650,10 @@
         <v>5013</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F63" s="4">
         <v>50003</v>
@@ -4654,10 +4662,10 @@
         <v>15</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K63" s="1">
         <v>14432</v>
@@ -4690,10 +4698,10 @@
         <v>5014</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F64" s="4">
         <v>50004</v>
@@ -4702,10 +4710,10 @@
         <v>15</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K64" s="1">
         <v>38484</v>
@@ -4738,10 +4746,10 @@
         <v>5015</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F65" s="4">
         <v>50005</v>
@@ -4750,10 +4758,10 @@
         <v>15</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K65" s="1">
         <v>-5260</v>
@@ -4786,10 +4794,10 @@
         <v>5016</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F66" s="4">
         <v>50006</v>
@@ -4798,10 +4806,10 @@
         <v>15</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K66" s="1">
         <v>6724</v>

</xml_diff>